<commit_message>
Add IA ground-truth crosscheck pipeline
Adds the IA evaluation pipeline artifacts: ground-truth conversion, discriminant classification, crosscheck reporting, pinfix diffing, and motor tracing. Also updates IA report docs, adds a crosscheck test suite, and applies UTF-8 console shims to the resolver scripts for Windows output safety.
</commit_message>
<xml_diff>
--- a/docs/reports/gold_templates/gold_IA_rotular.xlsx
+++ b/docs/reports/gold_templates/gold_IA_rotular.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Humberto\Documents\GitHub\GPT-Tutor-Generator\docs\reports\gold_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0067AE5A-0624-4D88-B0B2-59367827B4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9333302-8ABF-49EB-9D86-AE79D213F986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rotulagem" sheetId="1" r:id="rId1"/>
     <sheet name="Gabarito Subtopicos" sheetId="2" r:id="rId2"/>
+    <sheet name="Blocos" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="232">
   <si>
     <t>#</t>
   </si>
@@ -53,6 +54,12 @@
     <t>aula01 Introducao IA</t>
   </si>
   <si>
+    <t>01 — Plano de Ensino / Visão Geral da IA</t>
+  </si>
+  <si>
+    <t>alta</t>
+  </si>
+  <si>
     <t>IA Responsável</t>
   </si>
   <si>
@@ -77,6 +84,9 @@
     <t>Analise Exploratória dos Dados Exemplo 2</t>
   </si>
   <si>
+    <t>03 — Preparação de Dados / k-NN</t>
+  </si>
+  <si>
     <t>CaracteristicasDosDados.pdf</t>
   </si>
   <si>
@@ -89,6 +99,9 @@
     <t>Características dos Dados</t>
   </si>
   <si>
+    <t>02 — Introdução à ML / Tipos de Dados</t>
+  </si>
+  <si>
     <t>Introdução a ML.pdf</t>
   </si>
   <si>
@@ -113,6 +126,9 @@
     <t>Aprendizado Supervisionado Arvores De Decisao Duncan</t>
   </si>
   <si>
+    <t>07 — Regressão / Árvores de Decisão</t>
+  </si>
+  <si>
     <t>AprendizadoSupervisionado-Classificacao - kNN.pdf</t>
   </si>
   <si>
@@ -143,6 +159,9 @@
     <t>Introducao a redes neurais</t>
   </si>
   <si>
+    <t>04 — k-NN (exercícios) / Redes Neurais (intro)</t>
+  </si>
+  <si>
     <t>IntroducaoRedesNeurais_2023_02.pdf</t>
   </si>
   <si>
@@ -155,6 +174,9 @@
     <t>MLP</t>
   </si>
   <si>
+    <t>05 — Perceptron / MLP</t>
+  </si>
+  <si>
     <t>mlp_novaVersao.pdf</t>
   </si>
   <si>
@@ -191,6 +213,9 @@
     <t>Como analisar resultados Acc, Pr, Re e F1</t>
   </si>
   <si>
+    <t>06 — MLP (exercícios) / Métricas</t>
+  </si>
+  <si>
     <t>Como Analisar Resultados - SSE_comCorrecoes.pdf</t>
   </si>
   <si>
@@ -203,12 +228,21 @@
     <t>Inteligencia Artificial Aula 29 Aprendizagem de Maquina Medidas de avaliação</t>
   </si>
   <si>
+    <t>baixa</t>
+  </si>
+  <si>
     <t>agrupamento usando k-Means exemplo 1 (.ipynb).ipynb</t>
   </si>
   <si>
     <t>agrupamento usando k Means exemplo 1 (.ipynb)</t>
   </si>
   <si>
+    <t>08 — k-Means</t>
+  </si>
+  <si>
+    <t>Mesmo arquivo que o material "Como analisar resultados Acc, Pr, Re e F1.pdf"</t>
+  </si>
+  <si>
     <t>agrupamento usando k-Means exemplo 2 (.ipynb).ipynb</t>
   </si>
   <si>
@@ -227,6 +261,9 @@
     <t>Aprendizado Nao Supervisionado Agrupamento parte2</t>
   </si>
   <si>
+    <t>09 — Agrupamento Hierárquico / Dúvidas T1</t>
+  </si>
+  <si>
     <t>Artigo usando agrupamento.pdf</t>
   </si>
   <si>
@@ -257,18 +294,27 @@
     <t>AG feito em aula pelo Luca</t>
   </si>
   <si>
+    <t>13 — Algoritmos Genéticos (AG)</t>
+  </si>
+  <si>
     <t>Algoritmo Dijkstra.pdf</t>
   </si>
   <si>
     <t>Algoritmo Dijkstra</t>
   </si>
   <si>
+    <t>14 — Hill Climbing-SA / Dijkstra</t>
+  </si>
+  <si>
     <t>Algoritmo Genetico.pdf</t>
   </si>
   <si>
     <t>Algoritmo Genetico</t>
   </si>
   <si>
+    <t>12 — Busca Informada / Algoritmos Genéticos (AG)</t>
+  </si>
+  <si>
     <t>Cap. sobre Algoritmos Geneticos (Lacerda e outros).pdf</t>
   </si>
   <si>
@@ -287,6 +333,9 @@
     <t>Implementacao Minimax</t>
   </si>
   <si>
+    <t>15 — Minimax / Correção P1 / Dúvidas T2</t>
+  </si>
+  <si>
     <t>Introducao a busca informada.pdf</t>
   </si>
   <si>
@@ -332,12 +381,18 @@
     <t>Lista de Exercicios I</t>
   </si>
   <si>
+    <t>média</t>
+  </si>
+  <si>
     <t>lista1.pdf</t>
   </si>
   <si>
     <t>lista1</t>
   </si>
   <si>
+    <t>11 — Exercícios Gerais / Prova 1 (P1)</t>
+  </si>
+  <si>
     <t>P1_2024_02_IA.pdf</t>
   </si>
   <si>
@@ -353,6 +408,111 @@
     <t>Prova 1 2024 02</t>
   </si>
   <si>
+    <t xml:space="preserve">P2_IA_2024.pdf </t>
+  </si>
+  <si>
+    <t>Prova 2 2024 02</t>
+  </si>
+  <si>
+    <t>18 — Apresentação T2 / Prova P2</t>
+  </si>
+  <si>
+    <t>Agentes.pdf</t>
+  </si>
+  <si>
+    <t>Agentes IA</t>
+  </si>
+  <si>
+    <t>17 — Introdução a Agentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2_IA_2024_02_A_turma30.pdf </t>
+  </si>
+  <si>
+    <t>Prova 02 IA Turma 30</t>
+  </si>
+  <si>
+    <t>Análise Exploratória de Dados - Exemplo 1.ipynb</t>
+  </si>
+  <si>
+    <t>codigo</t>
+  </si>
+  <si>
+    <t>Analise Exploratoria / Prep. de Dados</t>
+  </si>
+  <si>
+    <t>Exemplo 2 k-NN (com IRIS.csv) - mais completo.ipynb</t>
+  </si>
+  <si>
+    <t>k-NN</t>
+  </si>
+  <si>
+    <t>Exemplo com k-NN.ipynb</t>
+  </si>
+  <si>
+    <t>Exercicio 2 - Solução com rede Perceptron (atualizado).ipynb</t>
+  </si>
+  <si>
+    <t>Perceptron</t>
+  </si>
+  <si>
+    <t>K-NN para Classificação Exemplo Cardio.ipynb</t>
+  </si>
+  <si>
+    <t>K-NN para Regressão exemplo IMC.ipynb</t>
+  </si>
+  <si>
+    <t>Rede Perceptron - Classificacao - Planta Iris.ipynb</t>
+  </si>
+  <si>
+    <t>Rede Perceptron - Classificacao de Cliente.ipynb</t>
+  </si>
+  <si>
+    <t>Rede Perceptron - Exemplo Atualizado.ipynb</t>
+  </si>
+  <si>
+    <t>Rede Perceptron - OR em Python.ipynb</t>
+  </si>
+  <si>
+    <t>Rede Perceptron - Reconhecendo Letras.ipynb</t>
+  </si>
+  <si>
+    <t>MLP - XOR.ipynb.ipynb</t>
+  </si>
+  <si>
+    <t>MLP Classificação - Inadimplência (normalização e GridSearchCV).ipynb</t>
+  </si>
+  <si>
+    <t>MLP Classificação - IRIS atualizado.ipynb</t>
+  </si>
+  <si>
+    <t>MLP Regressão - Cardio.ipynb</t>
+  </si>
+  <si>
+    <t>XOR - Backpropagation em python.ipynb</t>
+  </si>
+  <si>
+    <t>Exemplo 1 - Árvores de Decisão Classificação - Planta Iris.ipynb</t>
+  </si>
+  <si>
+    <t>Arvores de Decisao</t>
+  </si>
+  <si>
+    <t>Exemplo 2 - Arvores de Decisão - Regressão - Diabetes.ipynb</t>
+  </si>
+  <si>
+    <t>Exemplo Complementar - Classificação com Árvores de Decisão.ipynb</t>
+  </si>
+  <si>
+    <t>agrupamento hierarquico - exemplo 1.ipynb</t>
+  </si>
+  <si>
+    <t>Agrupamento Hierarquico</t>
+  </si>
+  <si>
+    <t>agrupamento hierarquico - exemplo 2 (use o dataset da planta IRIS).ipynb</t>
+  </si>
+  <si>
     <t>subtópico</t>
   </si>
   <si>
@@ -380,9 +540,6 @@
     <t>Roteiro+SARC</t>
   </si>
   <si>
-    <t>01 — Plano de Ensino / Visão Geral da IA</t>
-  </si>
-  <si>
     <t>Introdução à ML / Tipos de Dados</t>
   </si>
   <si>
@@ -392,9 +549,6 @@
     <t>ML / dados</t>
   </si>
   <si>
-    <t>02 — Introdução à ML / Tipos de Dados</t>
-  </si>
-  <si>
     <t>Preparação de Dados / k-NN</t>
   </si>
   <si>
@@ -404,9 +558,6 @@
     <t>dados / supervisionado</t>
   </si>
   <si>
-    <t>03 — Preparação de Dados / k-NN</t>
-  </si>
-  <si>
     <t>k-NN (exercícios) / Redes Neurais (intro)</t>
   </si>
   <si>
@@ -416,27 +567,18 @@
     <t>supervisionado</t>
   </si>
   <si>
-    <t>04 — k-NN (exercícios) / Redes Neurais (intro)</t>
-  </si>
-  <si>
     <t>Perceptron / MLP</t>
   </si>
   <si>
     <t>30/03, 01/04</t>
   </si>
   <si>
-    <t>05 — Perceptron / MLP</t>
-  </si>
-  <si>
     <t>MLP (exercícios) / Métricas</t>
   </si>
   <si>
     <t>06/04, 08/04</t>
   </si>
   <si>
-    <t>06 — MLP (exercícios) / Métricas</t>
-  </si>
-  <si>
     <t>Regressão / Árvores de Decisão</t>
   </si>
   <si>
@@ -446,9 +588,6 @@
     <t>Roteiro+SARC (13/04: SARC)</t>
   </si>
   <si>
-    <t>07 — Regressão / Árvores de Decisão</t>
-  </si>
-  <si>
     <t>k-Means</t>
   </si>
   <si>
@@ -461,18 +600,12 @@
     <t>SARC</t>
   </si>
   <si>
-    <t>08 — k-Means</t>
-  </si>
-  <si>
     <t>Agrupamento Hierárquico / Dúvidas T1</t>
   </si>
   <si>
     <t>27/04, 29/04</t>
   </si>
   <si>
-    <t>09 — Agrupamento Hierárquico / Dúvidas T1</t>
-  </si>
-  <si>
     <t>Apresentação T1</t>
   </si>
   <si>
@@ -494,9 +627,6 @@
     <t>avaliação</t>
   </si>
   <si>
-    <t>11 — Exercícios Gerais / Prova 1 (P1)</t>
-  </si>
-  <si>
     <t>Busca Informada / Algoritmos Genéticos (AG)</t>
   </si>
   <si>
@@ -509,9 +639,6 @@
     <t>Card S12 + mat</t>
   </si>
   <si>
-    <t>12 — Busca Informada / Algoritmos Genéticos (AG)</t>
-  </si>
-  <si>
     <t>Algoritmos Genéticos (AG)</t>
   </si>
   <si>
@@ -521,9 +648,6 @@
     <t>Card S13 + mat</t>
   </si>
   <si>
-    <t>13 — Algoritmos Genéticos (AG)</t>
-  </si>
-  <si>
     <t>Hill Climbing-SA / Dijkstra</t>
   </si>
   <si>
@@ -533,9 +657,6 @@
     <t>Roteiro (01/06) + Card S14</t>
   </si>
   <si>
-    <t>14 — Hill Climbing-SA / Dijkstra</t>
-  </si>
-  <si>
     <t>Minimax / Correção P1 / Dúvidas T2</t>
   </si>
   <si>
@@ -545,9 +666,6 @@
     <t>Card S15 + mat</t>
   </si>
   <si>
-    <t>15 — Minimax / Correção P1 / Dúvidas T2</t>
-  </si>
-  <si>
     <t>Busca (exercícios) / Introdução a Agentes</t>
   </si>
   <si>
@@ -569,9 +687,6 @@
     <t>agentes</t>
   </si>
   <si>
-    <t>17 — Introdução a Agentes</t>
-  </si>
-  <si>
     <t>Apresentação T2 / Prova P2</t>
   </si>
   <si>
@@ -581,9 +696,6 @@
     <t>trabalho / avaliação</t>
   </si>
   <si>
-    <t>18 — Apresentação T2 / Prova P2</t>
-  </si>
-  <si>
     <t>Prova PS / Atendimento-Divulgação</t>
   </si>
   <si>
@@ -606,36 +718,6 @@
   </si>
   <si>
     <t>não sei</t>
-  </si>
-  <si>
-    <t>alta</t>
-  </si>
-  <si>
-    <t>baixa</t>
-  </si>
-  <si>
-    <t>Mesmo arquivo que o material "Como analisar resultados Acc, Pr, Re e F1.pdf"</t>
-  </si>
-  <si>
-    <t>média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2_IA_2024.pdf </t>
-  </si>
-  <si>
-    <t>Prova 2 2024 02</t>
-  </si>
-  <si>
-    <t>Agentes.pdf</t>
-  </si>
-  <si>
-    <t>Agentes IA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2_IA_2024_02_A_turma30.pdf </t>
-  </si>
-  <si>
-    <t>Prova 02 IA Turma 30</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1088,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1055,10 +1137,10 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G2" s="6"/>
     </row>
@@ -1067,19 +1149,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>119</v>
-      </c>
       <c r="F3" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G3" s="6"/>
     </row>
@@ -1088,19 +1170,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G4" s="6"/>
     </row>
@@ -1109,19 +1191,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G5" s="6"/>
     </row>
@@ -1130,19 +1212,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G6" s="6"/>
     </row>
@@ -1151,19 +1233,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G7" s="6"/>
     </row>
@@ -1172,19 +1254,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>123</v>
+        <v>25</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G8" s="6"/>
     </row>
@@ -1193,19 +1275,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>123</v>
+        <v>25</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G9" s="6"/>
     </row>
@@ -1214,19 +1296,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>123</v>
-      </c>
       <c r="F10" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G10" s="6"/>
     </row>
@@ -1235,38 +1317,38 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F11" s="5"/>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>141</v>
+        <v>34</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G12" s="6"/>
     </row>
@@ -1275,19 +1357,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G13" s="6"/>
     </row>
@@ -1296,19 +1378,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G14" s="6"/>
     </row>
@@ -1317,19 +1399,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>141</v>
-      </c>
       <c r="F15" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G15" s="6"/>
     </row>
@@ -1338,19 +1420,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G16" s="6"/>
     </row>
@@ -1359,19 +1441,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G17" s="6"/>
     </row>
@@ -1380,19 +1462,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G18" s="6"/>
     </row>
@@ -1401,19 +1483,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G19" s="6"/>
     </row>
@@ -1422,19 +1504,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G20" s="6"/>
     </row>
@@ -1443,19 +1525,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G21" s="6"/>
     </row>
@@ -1464,19 +1546,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G22" s="6"/>
     </row>
@@ -1485,19 +1567,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>134</v>
-      </c>
       <c r="F23" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G23" s="6"/>
     </row>
@@ -1506,19 +1588,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G24" s="6"/>
     </row>
@@ -1527,19 +1609,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G25" s="6"/>
     </row>
@@ -1548,64 +1630,64 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>196</v>
+        <v>68</v>
       </c>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1613,61 +1695,61 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G29" s="6"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G31" s="6"/>
     </row>
@@ -1676,19 +1758,19 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G32" s="6"/>
     </row>
@@ -1697,19 +1779,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="5" t="s">
-        <v>146</v>
-      </c>
       <c r="F33" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G33" s="6"/>
     </row>
@@ -1718,19 +1800,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G34" s="6"/>
     </row>
@@ -1739,19 +1821,19 @@
         <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G35" s="6"/>
     </row>
@@ -1760,19 +1842,19 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G36" s="6"/>
     </row>
@@ -1781,19 +1863,19 @@
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>170</v>
+        <v>93</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G37" s="6"/>
     </row>
@@ -1802,40 +1884,40 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G39" s="6"/>
     </row>
@@ -1844,19 +1926,19 @@
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>170</v>
+        <v>93</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G40" s="6"/>
     </row>
@@ -1865,19 +1947,19 @@
         <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G41" s="6"/>
     </row>
@@ -1886,19 +1968,19 @@
         <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G42" s="6"/>
     </row>
@@ -1907,19 +1989,19 @@
         <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G43" s="6"/>
     </row>
@@ -1928,17 +2010,17 @@
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G44" s="6"/>
     </row>
@@ -1947,19 +2029,19 @@
         <v>44</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G45" s="6"/>
     </row>
@@ -1968,38 +2050,38 @@
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>170</v>
+        <v>93</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G47" s="6"/>
     </row>
@@ -2008,19 +2090,19 @@
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>198</v>
+        <v>119</v>
       </c>
       <c r="G48" s="6"/>
     </row>
@@ -2029,19 +2111,19 @@
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>198</v>
+        <v>119</v>
       </c>
       <c r="G49" s="6"/>
     </row>
@@ -2050,19 +2132,19 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>198</v>
+        <v>119</v>
       </c>
       <c r="G50" s="6"/>
     </row>
@@ -2071,19 +2153,19 @@
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>198</v>
+        <v>119</v>
       </c>
       <c r="G51" s="6"/>
     </row>
@@ -2092,19 +2174,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>199</v>
+        <v>128</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>200</v>
+        <v>129</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>186</v>
+        <v>130</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G52" s="6"/>
     </row>
@@ -2113,19 +2195,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>201</v>
+        <v>131</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>202</v>
+        <v>132</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>182</v>
+        <v>133</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G53" s="6"/>
     </row>
@@ -2134,30 +2216,482 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>203</v>
+        <v>134</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>204</v>
+        <v>135</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>186</v>
+        <v>130</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="G54" s="6"/>
     </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>136</v>
+      </c>
+      <c r="C55" t="s">
+        <v>137</v>
+      </c>
+      <c r="D55" t="s">
+        <v>138</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G55" s="6"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>139</v>
+      </c>
+      <c r="C56" t="s">
+        <v>137</v>
+      </c>
+      <c r="D56" t="s">
+        <v>140</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" s="6"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>141</v>
+      </c>
+      <c r="C57" t="s">
+        <v>137</v>
+      </c>
+      <c r="D57" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G57" s="6"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>142</v>
+      </c>
+      <c r="C58" t="s">
+        <v>137</v>
+      </c>
+      <c r="D58" t="s">
+        <v>143</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G58" s="6"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>144</v>
+      </c>
+      <c r="C59" t="s">
+        <v>137</v>
+      </c>
+      <c r="D59" t="s">
+        <v>140</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G59" s="6"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>145</v>
+      </c>
+      <c r="C60" t="s">
+        <v>137</v>
+      </c>
+      <c r="D60" t="s">
+        <v>140</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G60" s="6"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>146</v>
+      </c>
+      <c r="C61" t="s">
+        <v>137</v>
+      </c>
+      <c r="D61" t="s">
+        <v>143</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G61" s="6"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>147</v>
+      </c>
+      <c r="C62" t="s">
+        <v>137</v>
+      </c>
+      <c r="D62" t="s">
+        <v>143</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G62" s="6"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>148</v>
+      </c>
+      <c r="C63" t="s">
+        <v>137</v>
+      </c>
+      <c r="D63" t="s">
+        <v>143</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F63" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G63" s="6"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>149</v>
+      </c>
+      <c r="C64" t="s">
+        <v>137</v>
+      </c>
+      <c r="D64" t="s">
+        <v>143</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G64" s="6"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>150</v>
+      </c>
+      <c r="C65" t="s">
+        <v>137</v>
+      </c>
+      <c r="D65" t="s">
+        <v>143</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G65" s="6"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>151</v>
+      </c>
+      <c r="C66" t="s">
+        <v>137</v>
+      </c>
+      <c r="D66" t="s">
+        <v>49</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" s="6"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>152</v>
+      </c>
+      <c r="C67" t="s">
+        <v>137</v>
+      </c>
+      <c r="D67" t="s">
+        <v>49</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" s="6"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>153</v>
+      </c>
+      <c r="C68" t="s">
+        <v>137</v>
+      </c>
+      <c r="D68" t="s">
+        <v>49</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G68" s="6"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>154</v>
+      </c>
+      <c r="C69" t="s">
+        <v>137</v>
+      </c>
+      <c r="D69" t="s">
+        <v>49</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G69" s="6"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>155</v>
+      </c>
+      <c r="C70" t="s">
+        <v>137</v>
+      </c>
+      <c r="D70" t="s">
+        <v>49</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G70" s="6"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>156</v>
+      </c>
+      <c r="C71" t="s">
+        <v>137</v>
+      </c>
+      <c r="D71" t="s">
+        <v>157</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G71" s="6"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>158</v>
+      </c>
+      <c r="C72" t="s">
+        <v>137</v>
+      </c>
+      <c r="D72" t="s">
+        <v>157</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G72" s="6"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>159</v>
+      </c>
+      <c r="C73" t="s">
+        <v>137</v>
+      </c>
+      <c r="D73" t="s">
+        <v>157</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G73" s="6"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>160</v>
+      </c>
+      <c r="C74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D74" t="s">
+        <v>161</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G74" s="6"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>162</v>
+      </c>
+      <c r="C75" t="s">
+        <v>137</v>
+      </c>
+      <c r="D75" t="s">
+        <v>161</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G75" s="6"/>
+    </row>
   </sheetData>
-  <sheetProtection formatColumns="0" selectLockedCells="1" sort="0" autoFilter="0" selectUnlockedCells="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" prompt="Sua confiança na resposta." sqref="F2:F54" xr:uid="{E94B99D0-738B-485C-AFA5-91432A88608B}">
+    <dataValidation type="list" allowBlank="1" prompt="Sua confiança na resposta." sqref="F2:F75" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"alta,média,baixa"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" promptTitle="bloco_correto" prompt="Escolha o bloco correto da lista." xr:uid="{00000000-0002-0000-0000-000001000000}">
+          <x14:formula1>
+            <xm:f>Blocos!$A$1:$A$16</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E75</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2179,19 +2713,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>165</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>166</v>
       </c>
       <c r="F1" t="s">
-        <v>114</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -2199,19 +2733,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>115</v>
+        <v>168</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>116</v>
+        <v>169</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>117</v>
+        <v>170</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F2" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -2219,19 +2753,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>121</v>
+        <v>173</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F3" t="s">
-        <v>123</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -2239,19 +2773,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>124</v>
+        <v>175</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>125</v>
+        <v>176</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>126</v>
+        <v>177</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F4" t="s">
-        <v>127</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -2259,19 +2793,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>128</v>
+        <v>178</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>129</v>
+        <v>179</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F5" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -2279,19 +2813,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F6" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -2299,39 +2833,39 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>135</v>
+        <v>183</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F7" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>138</v>
+        <v>185</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>139</v>
+        <v>186</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="F8" t="s">
-        <v>141</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -2339,19 +2873,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>143</v>
+        <v>189</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="F9" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -2359,19 +2893,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>147</v>
+        <v>192</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>148</v>
+        <v>193</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F10" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -2379,19 +2913,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>150</v>
+        <v>194</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>151</v>
+        <v>195</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="F11" t="s">
-        <v>153</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -2399,39 +2933,39 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>154</v>
+        <v>198</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>156</v>
+        <v>200</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F12" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>158</v>
+        <v>201</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>159</v>
+        <v>202</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>161</v>
+        <v>204</v>
       </c>
       <c r="F13" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -2439,39 +2973,39 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>163</v>
+        <v>205</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>164</v>
+        <v>206</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>165</v>
+        <v>207</v>
       </c>
       <c r="F14" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>167</v>
+        <v>208</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>168</v>
+        <v>209</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>169</v>
+        <v>210</v>
       </c>
       <c r="F15" t="s">
-        <v>170</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -2479,19 +3013,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="F16" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -2499,19 +3033,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>176</v>
+        <v>215</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>177</v>
+        <v>216</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="F17" t="s">
-        <v>178</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -2519,19 +3053,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>179</v>
+        <v>218</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="F18" t="s">
-        <v>182</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -2539,19 +3073,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>183</v>
+        <v>221</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>184</v>
+        <v>222</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>185</v>
+        <v>223</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="F19" t="s">
-        <v>186</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -2559,19 +3093,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>187</v>
+        <v>224</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>188</v>
+        <v>225</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>156</v>
+        <v>200</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="F20" t="s">
-        <v>189</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -2579,19 +3113,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>190</v>
+        <v>227</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>145</v>
-      </c>
       <c r="F21" t="s">
-        <v>192</v>
+        <v>229</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2601,7 +3135,7 @@
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" t="s">
-        <v>193</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -2611,7 +3145,97 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" t="s">
-        <v>194</v>
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
style(gold): uniformiza coluna tipo do IA/ES2 (file_type)
Reescreve so a coluna 'tipo' dos golds ja rotulados (IA/ES2) do file_type do
manifest (+ fallback por extensao nas linhas unjoined), pra bater com o padrao
file_type dos demais. Rotulos/obs/dropdowns preservados; ground_truth_IA
regenera byte-identico (tipo nao e lido pelo crosswalk). Cosmetico.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRQpbp1NNFwNrJaHsq41XT
</commit_message>
<xml_diff>
--- a/docs/reports/gold_templates/gold_IA_rotular.xlsx
+++ b/docs/reports/gold_templates/gold_IA_rotular.xlsx
@@ -540,7 +540,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>link</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>link</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>material</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>material</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">

</xml_diff>